<commit_message>
:recycle: Refactoring code. 适配最新 V5 UI
</commit_message>
<xml_diff>
--- a/pigx-upms/pigx-upms-biz/src/main/resources/file/dept.xlsx
+++ b/pigx-upms/pigx-upms-biz/src/main/resources/file/dept.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wfu7326\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pigxProject\pigx-boot\pigx-upms\pigx-upms-biz\src\main\resources\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE8C7C76-B37A-4303-8731-E63EBB79B6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E4BC8CC-A6A3-47EA-9564-6C1877BCC420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,10 +31,11 @@
     <t>排序值</t>
   </si>
   <si>
-    <t>跟部门</t>
+    <t>山东</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>山东</t>
+    <t>根部门</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -42,7 +43,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -71,6 +72,12 @@
       <sz val="11"/>
       <name val="宋体"/>
       <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -116,7 +123,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -125,6 +132,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -458,12 +466,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
+    <row r="2" spans="1:3" ht="16.5">
+      <c r="A2" s="4" t="s">
+        <v>4</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>

</xml_diff>